<commit_message>
Exclude test accounts from white-label partner banner report
Removed tututut33333555, jkjkjkjkjj, Tester, Testering from Excel and PDF

Co-authored-by: paladuguraj <paladuguraj@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/white-label-partner-banners.xlsx
+++ b/reports/white-label-partner-banners.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F32"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1039,89 +1039,9 @@
         <v>No</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>tututut33333555</v>
-      </c>
-      <c r="B33" t="str">
-        <v/>
-      </c>
-      <c r="C33" t="str">
-        <v/>
-      </c>
-      <c r="D33" t="str">
-        <v/>
-      </c>
-      <c r="E33" t="str">
-        <v>5fc7682d3367c390f4c08dc91e5c7b64</v>
-      </c>
-      <c r="F33" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>jkjkjkjkjj</v>
-      </c>
-      <c r="B34" t="str">
-        <v/>
-      </c>
-      <c r="C34" t="str">
-        <v/>
-      </c>
-      <c r="D34" t="str">
-        <v/>
-      </c>
-      <c r="E34" t="str">
-        <v>8817a0e93367c390f4c08dc91e5c7b15</v>
-      </c>
-      <c r="F34" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v>Tester</v>
-      </c>
-      <c r="B35" t="str">
-        <v/>
-      </c>
-      <c r="C35" t="str">
-        <v/>
-      </c>
-      <c r="D35" t="str">
-        <v/>
-      </c>
-      <c r="E35" t="str">
-        <v>b2762c693367c390f4c08dc91e5c7bf1</v>
-      </c>
-      <c r="F35" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>Testering</v>
-      </c>
-      <c r="B36" t="str">
-        <v/>
-      </c>
-      <c r="C36" t="str">
-        <v/>
-      </c>
-      <c r="D36" t="str">
-        <v/>
-      </c>
-      <c r="E36" t="str">
-        <v>d9e6a8a93367c390f4c08dc91e5c7b65</v>
-      </c>
-      <c r="F36" t="str">
-        <v>No</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F32"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Expand banner report to all 39 white-label partner accounts
- Add 5 CSV accounts confirmed without banner images
- Add 3 CSV accounts with banner images (WarpSpeed, Aurora, Bedroc) with fetched file size/type/dimensions
- Total: 39 accounts (31 with banner, 8 without)

Co-authored-by: paladuguraj <paladuguraj@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/white-label-partner-banners.xlsx
+++ b/reports/white-label-partner-banners.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F40"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -981,67 +981,227 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Maverick Speed</v>
+        <v>WarpSpeed Group LLC</v>
       </c>
       <c r="B30" t="str">
-        <v/>
-      </c>
-      <c r="C30" t="str">
-        <v/>
+        <v>image/png</v>
+      </c>
+      <c r="C30">
+        <v>11569</v>
       </c>
       <c r="D30" t="str">
-        <v/>
+        <v>PNG image data, 250 x 100, 8-bit/color RGBA, non-interlaced</v>
       </c>
       <c r="E30" t="str">
-        <v>25510419fbf5aed04c95fc287befdc1d</v>
+        <v>97a7e8cb3b69bed0a9d88aac24e45a11</v>
       </c>
       <c r="F30" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>DSI Distributing Inc.</v>
+        <v>Aurora Communications LLC</v>
       </c>
       <c r="B31" t="str">
-        <v/>
-      </c>
-      <c r="C31" t="str">
-        <v/>
+        <v>image/jpeg</v>
+      </c>
+      <c r="C31">
+        <v>6360</v>
       </c>
       <c r="D31" t="str">
-        <v/>
+        <v>JPEG image data, 326 x 65, components 3</v>
       </c>
       <c r="E31" t="str">
-        <v>2a734f572bf06e101afef5b36e91bf00</v>
+        <v>47bcd2ab3bcae2509f13571864e45a8b</v>
       </c>
       <c r="F31" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
+        <v>Bedroc Partner</v>
+      </c>
+      <c r="B32" t="str">
+        <v>image/png</v>
+      </c>
+      <c r="C32">
+        <v>28288</v>
+      </c>
+      <c r="D32" t="str">
+        <v>PNG image data, 194 x 175, 8-bit/color RGBA, non-interlaced</v>
+      </c>
+      <c r="E32" t="str">
+        <v>c8dc4a2adbd950100eea89584b96197c</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Maverick Speed</v>
+      </c>
+      <c r="B33" t="str">
+        <v/>
+      </c>
+      <c r="C33" t="str">
+        <v/>
+      </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
+      <c r="E33" t="str">
+        <v>25510419fbf5aed04c95fc287befdc1d</v>
+      </c>
+      <c r="F33" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>DSI Distributing Inc.</v>
+      </c>
+      <c r="B34" t="str">
+        <v/>
+      </c>
+      <c r="C34" t="str">
+        <v/>
+      </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
+      <c r="E34" t="str">
+        <v>2a734f572bf06e101afef5b36e91bf00</v>
+      </c>
+      <c r="F34" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
         <v>LevelBlue</v>
       </c>
-      <c r="B32" t="str">
-        <v/>
-      </c>
-      <c r="C32" t="str">
-        <v/>
-      </c>
-      <c r="D32" t="str">
-        <v/>
-      </c>
-      <c r="E32" t="str">
+      <c r="B35" t="str">
+        <v/>
+      </c>
+      <c r="C35" t="str">
+        <v/>
+      </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
+      <c r="E35" t="str">
         <v>4a8fd0722b3f3a501afef5b36e91bfc6</v>
       </c>
-      <c r="F32" t="str">
+      <c r="F35" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Blue Plains Technology</v>
+      </c>
+      <c r="B36" t="str">
+        <v/>
+      </c>
+      <c r="C36" t="str">
+        <v/>
+      </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
+      <c r="E36" t="str">
+        <v>7bfe925b3313c390d814e4b32d5c7b6f</v>
+      </c>
+      <c r="F36" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Itecs</v>
+      </c>
+      <c r="B37" t="str">
+        <v/>
+      </c>
+      <c r="C37" t="str">
+        <v/>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v>7f6f5adb3313c390d814e4b32d5c7b0e</v>
+      </c>
+      <c r="F37" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Sora Partners</v>
+      </c>
+      <c r="B38" t="str">
+        <v/>
+      </c>
+      <c r="C38" t="str">
+        <v/>
+      </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
+      <c r="E38" t="str">
+        <v>84ef529f3313c390d814e4b32d5c7b21</v>
+      </c>
+      <c r="F38" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Triton Networks</v>
+      </c>
+      <c r="B39" t="str">
+        <v/>
+      </c>
+      <c r="C39" t="str">
+        <v/>
+      </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
+      <c r="E39" t="str">
+        <v>7d106edf3313c390d814e4b32d5c7bf9</v>
+      </c>
+      <c r="F39" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Xentegra</v>
+      </c>
+      <c r="B40" t="str">
+        <v/>
+      </c>
+      <c r="C40" t="str">
+        <v/>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v>559d5b963bd343509f13571864e45a0e</v>
+      </c>
+      <c r="F40" t="str">
         <v>No</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F40"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>